<commit_message>
Exclude 'Assigned' status from Worked; add notes sheet; consistent Direct LP wording
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014mYQKy48Wu36t4nGVjPjP9
</commit_message>
<xml_diff>
--- a/outputs/Monthly_Lead_Report_Oct2026_backing.xlsx
+++ b/outputs/Monthly_Lead_Report_Oct2026_backing.xlsx
@@ -12,14 +12,15 @@
     <sheet name="Exact counts" sheetId="3" r:id="rId3"/>
     <sheet name="Data checks" sheetId="4" r:id="rId4"/>
     <sheet name="Brand mapping used" sheetId="5" r:id="rId5"/>
-    <sheet name="Status counts" sheetId="6" r:id="rId6"/>
+    <sheet name="Notes" sheetId="6" r:id="rId6"/>
+    <sheet name="Status counts" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="169">
   <si>
     <t>Brand</t>
   </si>
@@ -132,7 +133,7 @@
     <t>28,449</t>
   </si>
   <si>
-    <t>25.16K</t>
+    <t>25.15K</t>
   </si>
   <si>
     <t>3.35K</t>
@@ -201,6 +202,9 @@
     <t>new_lead</t>
   </si>
   <si>
+    <t>assigned_status_not_worked</t>
+  </si>
+  <si>
     <t>connected</t>
   </si>
   <si>
@@ -436,6 +440,27 @@
   </si>
   <si>
     <t>Tarzan Nature Retreat</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Period: Created On 1 Oct 00:00 to 28 Oct 23:59:59 2026; both exports combined; de-duplicated on Lead id.</t>
+  </si>
+  <si>
+    <t>Counts are lead records (TeleCRM rows), not unique phone numbers; some phones appear in several leads/brands.</t>
+  </si>
+  <si>
+    <t>Any Brand starting FW_/FW- is the separate FW (Franchise World) brand.</t>
+  </si>
+  <si>
+    <t>Kabego Rental counted under EBG Rental; Realty and blank brands under Other / Unmapped.</t>
+  </si>
+  <si>
+    <t>Worked = all statuses except New Lead and Assigned. Quality Pipeline = Qualified, Details Shared, Meeting Scheduled/Conducted, Negotiation, Token Received.</t>
+  </si>
+  <si>
+    <t>Won = Token Received (CRM has no Won status). Direct LP Meetings and MIB Closures are not in the exports.</t>
   </si>
   <si>
     <t>Status</t>
@@ -1334,7 +1359,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1358,7 +1383,7 @@
         <v>58</v>
       </c>
       <c r="B3">
-        <v>25162</v>
+        <v>25152</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1374,7 +1399,7 @@
         <v>60</v>
       </c>
       <c r="B5">
-        <v>3353</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1382,7 +1407,7 @@
         <v>61</v>
       </c>
       <c r="B6">
-        <v>3973</v>
+        <v>3353</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1390,7 +1415,7 @@
         <v>62</v>
       </c>
       <c r="B7">
-        <v>1863</v>
+        <v>3973</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1398,7 +1423,7 @@
         <v>63</v>
       </c>
       <c r="B8">
-        <v>457</v>
+        <v>1863</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1406,7 +1431,7 @@
         <v>64</v>
       </c>
       <c r="B9">
-        <v>172</v>
+        <v>457</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1414,7 +1439,7 @@
         <v>65</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>172</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -1430,7 +1455,7 @@
         <v>67</v>
       </c>
       <c r="B12">
-        <v>6323</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -1438,7 +1463,7 @@
         <v>68</v>
       </c>
       <c r="B13">
-        <v>26137</v>
+        <v>6323</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -1446,6 +1471,14 @@
         <v>69</v>
       </c>
       <c r="B14">
+        <v>26137</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15">
         <v>285</v>
       </c>
     </row>
@@ -1461,15 +1494,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B2">
         <v>39103</v>
@@ -1477,7 +1510,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B3">
         <v>28451</v>
@@ -1485,7 +1518,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -1503,10 +1536,10 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1517,7 +1550,7 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C2">
         <v>3021</v>
@@ -1528,7 +1561,7 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C3">
         <v>61</v>
@@ -1550,7 +1583,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C5">
         <v>163</v>
@@ -1561,7 +1594,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C6">
         <v>646</v>
@@ -1572,7 +1605,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C7">
         <v>326</v>
@@ -1583,7 +1616,7 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1605,7 +1638,7 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C10">
         <v>2</v>
@@ -1616,7 +1649,7 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C11">
         <v>1521</v>
@@ -1627,7 +1660,7 @@
         <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C12">
         <v>572</v>
@@ -1638,7 +1671,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C13">
         <v>66</v>
@@ -1649,7 +1682,7 @@
         <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C14">
         <v>1017</v>
@@ -1660,7 +1693,7 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C15">
         <v>350</v>
@@ -1693,7 +1726,7 @@
         <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C18">
         <v>46</v>
@@ -1704,7 +1737,7 @@
         <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C19">
         <v>61</v>
@@ -1715,7 +1748,7 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C20">
         <v>9112</v>
@@ -1737,7 +1770,7 @@
         <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C22">
         <v>211</v>
@@ -1748,7 +1781,7 @@
         <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C23">
         <v>69</v>
@@ -1759,7 +1792,7 @@
         <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C24">
         <v>30</v>
@@ -1770,7 +1803,7 @@
         <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C25">
         <v>60</v>
@@ -1781,7 +1814,7 @@
         <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C26">
         <v>6</v>
@@ -1792,7 +1825,7 @@
         <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C27">
         <v>34</v>
@@ -1803,7 +1836,7 @@
         <v>12</v>
       </c>
       <c r="B28" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C28">
         <v>2</v>
@@ -1814,7 +1847,7 @@
         <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C29">
         <v>26</v>
@@ -1825,7 +1858,7 @@
         <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C30">
         <v>18</v>
@@ -1836,7 +1869,7 @@
         <v>12</v>
       </c>
       <c r="B31" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C31">
         <v>7</v>
@@ -1847,7 +1880,7 @@
         <v>12</v>
       </c>
       <c r="B32" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C32">
         <v>2</v>
@@ -1858,7 +1891,7 @@
         <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C33">
         <v>14</v>
@@ -1869,7 +1902,7 @@
         <v>12</v>
       </c>
       <c r="B34" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C34">
         <v>4</v>
@@ -1880,7 +1913,7 @@
         <v>12</v>
       </c>
       <c r="B35" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C35">
         <v>56</v>
@@ -1891,7 +1924,7 @@
         <v>12</v>
       </c>
       <c r="B36" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -1902,7 +1935,7 @@
         <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -1913,7 +1946,7 @@
         <v>12</v>
       </c>
       <c r="B38" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C38">
         <v>2</v>
@@ -1924,7 +1957,7 @@
         <v>12</v>
       </c>
       <c r="B39" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C39">
         <v>12</v>
@@ -1935,7 +1968,7 @@
         <v>12</v>
       </c>
       <c r="B40" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C40">
         <v>63</v>
@@ -1946,7 +1979,7 @@
         <v>12</v>
       </c>
       <c r="B41" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C41">
         <v>33</v>
@@ -1957,7 +1990,7 @@
         <v>12</v>
       </c>
       <c r="B42" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C42">
         <v>2</v>
@@ -1968,7 +2001,7 @@
         <v>12</v>
       </c>
       <c r="B43" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C43">
         <v>24</v>
@@ -1979,7 +2012,7 @@
         <v>12</v>
       </c>
       <c r="B44" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C44">
         <v>2</v>
@@ -1990,7 +2023,7 @@
         <v>12</v>
       </c>
       <c r="B45" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C45">
         <v>18</v>
@@ -2001,7 +2034,7 @@
         <v>12</v>
       </c>
       <c r="B46" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C46">
         <v>59</v>
@@ -2012,7 +2045,7 @@
         <v>12</v>
       </c>
       <c r="B47" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C47">
         <v>7</v>
@@ -2023,7 +2056,7 @@
         <v>12</v>
       </c>
       <c r="B48" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C48">
         <v>246</v>
@@ -2034,7 +2067,7 @@
         <v>12</v>
       </c>
       <c r="B49" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C49">
         <v>11</v>
@@ -2045,7 +2078,7 @@
         <v>12</v>
       </c>
       <c r="B50" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C50">
         <v>161</v>
@@ -2056,7 +2089,7 @@
         <v>12</v>
       </c>
       <c r="B51" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C51">
         <v>82</v>
@@ -2067,7 +2100,7 @@
         <v>12</v>
       </c>
       <c r="B52" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C52">
         <v>21</v>
@@ -2078,7 +2111,7 @@
         <v>12</v>
       </c>
       <c r="B53" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C53">
         <v>152</v>
@@ -2089,7 +2122,7 @@
         <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C54">
         <v>40</v>
@@ -2100,7 +2133,7 @@
         <v>12</v>
       </c>
       <c r="B55" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C55">
         <v>16</v>
@@ -2111,7 +2144,7 @@
         <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C56">
         <v>52</v>
@@ -2122,7 +2155,7 @@
         <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C57">
         <v>18</v>
@@ -2133,7 +2166,7 @@
         <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C58">
         <v>201</v>
@@ -2155,7 +2188,7 @@
         <v>11</v>
       </c>
       <c r="B60" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C60">
         <v>285</v>
@@ -2166,7 +2199,7 @@
         <v>15</v>
       </c>
       <c r="B61" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C61">
         <v>1808</v>
@@ -2188,7 +2221,7 @@
         <v>15</v>
       </c>
       <c r="B63" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C63">
         <v>151</v>
@@ -2199,7 +2232,7 @@
         <v>13</v>
       </c>
       <c r="B64" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C64">
         <v>811</v>
@@ -2210,7 +2243,7 @@
         <v>13</v>
       </c>
       <c r="B65" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C65">
         <v>90</v>
@@ -2221,7 +2254,7 @@
         <v>21</v>
       </c>
       <c r="B66" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C66">
         <v>250</v>
@@ -2232,7 +2265,7 @@
         <v>21</v>
       </c>
       <c r="B67" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C67">
         <v>117</v>
@@ -2243,7 +2276,7 @@
         <v>21</v>
       </c>
       <c r="B68" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C68">
         <v>430</v>
@@ -2254,7 +2287,7 @@
         <v>14</v>
       </c>
       <c r="B69" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C69">
         <v>1</v>
@@ -2265,7 +2298,7 @@
         <v>7</v>
       </c>
       <c r="B70" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C70">
         <v>244</v>
@@ -2278,12 +2311,57 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>146</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -2291,7 +2369,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="B2">
         <v>6180</v>
@@ -2299,7 +2377,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="B3">
         <v>5707</v>
@@ -2307,7 +2385,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="B4">
         <v>3353</v>
@@ -2315,7 +2393,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="B5">
         <v>3287</v>
@@ -2323,7 +2401,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B6">
         <v>2287</v>
@@ -2331,7 +2409,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="B7">
         <v>1863</v>
@@ -2339,7 +2417,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B8">
         <v>1651</v>
@@ -2347,7 +2425,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="B9">
         <v>1186</v>
@@ -2355,7 +2433,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B10">
         <v>847</v>
@@ -2363,7 +2441,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="B11">
         <v>772</v>
@@ -2371,7 +2449,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="B12">
         <v>528</v>
@@ -2379,7 +2457,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="B13">
         <v>285</v>
@@ -2387,7 +2465,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="B14">
         <v>166</v>
@@ -2395,7 +2473,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="B15">
         <v>154</v>
@@ -2403,7 +2481,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="B16">
         <v>143</v>
@@ -2411,7 +2489,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="B17">
         <v>19</v>
@@ -2427,7 +2505,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="B19">
         <v>6</v>
@@ -2435,7 +2513,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="B20">
         <v>2</v>
@@ -2443,7 +2521,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -2451,7 +2529,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="B22">
         <v>1</v>
@@ -2459,7 +2537,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B23">
         <v>1</v>

</xml_diff>